<commit_message>
Add October story screenshots to tracking sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016oX5BAioULTkYoqv5bsGKi
</commit_message>
<xml_diff>
--- a/sns_tracking/SNS記録シート.xlsx
+++ b/sns_tracking/SNS記録シート.xlsx
@@ -25,10 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="166" formatCode="m/d"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="165" formatCode="m/d"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -105,12 +104,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,7 +118,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,7 +137,16 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -224,6 +232,411 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>4</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1400175" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>5</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1400175" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>6</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1400175" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>7</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>8</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1381125" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>9</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1381125" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>10</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1381125" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>11</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1381125" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>12</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>13</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>14</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>15</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1371600" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>16</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1371600" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>17</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>18</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>19</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1390650" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -565,7 +978,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="13" t="n">
         <v>46296</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -583,7 +996,7 @@
       <c r="G2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="13" t="n">
         <v>46297</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -601,7 +1014,7 @@
       <c r="G3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="14" t="n">
         <v>46298</v>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -619,7 +1032,7 @@
       <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="14" t="n">
         <v>46299</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -637,7 +1050,7 @@
       <c r="G5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="13" t="n">
         <v>46300</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -655,7 +1068,7 @@
       <c r="G6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="13" t="n">
         <v>46301</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -673,7 +1086,7 @@
       <c r="G7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="13" t="n">
         <v>46302</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -691,7 +1104,7 @@
       <c r="G8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="13" t="n">
         <v>46303</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -709,7 +1122,7 @@
       <c r="G9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="13" t="n">
         <v>46304</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -727,7 +1140,7 @@
       <c r="G10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="14" t="n">
         <v>46305</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -745,7 +1158,7 @@
       <c r="G11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="14" t="n">
         <v>46306</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -763,7 +1176,7 @@
       <c r="G12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="13" t="n">
         <v>46307</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -781,7 +1194,7 @@
       <c r="G13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="13" t="n">
         <v>46308</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -799,7 +1212,7 @@
       <c r="G14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="13" t="n">
         <v>46309</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -817,7 +1230,7 @@
       <c r="G15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="13" t="n">
         <v>46310</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -835,7 +1248,7 @@
       <c r="G16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="13" t="n">
         <v>46311</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -853,7 +1266,7 @@
       <c r="G17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="14" t="n">
         <v>46312</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -871,7 +1284,7 @@
       <c r="G18" s="7" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="14" t="n">
         <v>46313</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -889,7 +1302,7 @@
       <c r="G19" s="7" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="13" t="n">
         <v>46314</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -907,7 +1320,7 @@
       <c r="G20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="13" t="n">
         <v>46315</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -925,7 +1338,7 @@
       <c r="G21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="13" t="n">
         <v>46316</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -943,7 +1356,7 @@
       <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="13" t="n">
         <v>46317</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -961,7 +1374,7 @@
       <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="13" t="n">
         <v>46318</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -979,7 +1392,7 @@
       <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="14" t="n">
         <v>46319</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -997,7 +1410,7 @@
       <c r="G25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="14" t="n">
         <v>46320</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1015,7 +1428,7 @@
       <c r="G26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="13" t="n">
         <v>46321</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1033,7 +1446,7 @@
       <c r="G27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="13" t="n">
         <v>46322</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1051,7 +1464,7 @@
       <c r="G28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="13" t="n">
         <v>46323</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1069,7 +1482,7 @@
       <c r="G29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="13" t="n">
         <v>46324</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1087,7 +1500,7 @@
       <c r="G30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="13" t="n">
         <v>46325</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1105,7 +1518,7 @@
       <c r="G31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="14" t="n">
         <v>46326</v>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1123,7 +1536,7 @@
       <c r="G32" s="7" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="14" t="n">
         <v>46327</v>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -1141,7 +1554,7 @@
       <c r="G33" s="7" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="13" t="n">
         <v>46328</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1159,7 +1572,7 @@
       <c r="G34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="13" t="n">
         <v>46329</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1177,7 +1590,7 @@
       <c r="G35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="13" t="n">
         <v>46330</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1195,7 +1608,7 @@
       <c r="G36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="13" t="n">
         <v>46331</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1213,7 +1626,7 @@
       <c r="G37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="13" t="n">
         <v>46332</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1231,7 +1644,7 @@
       <c r="G38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="14" t="n">
         <v>46333</v>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1249,7 +1662,7 @@
       <c r="G39" s="7" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="14" t="n">
         <v>46334</v>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -1267,7 +1680,7 @@
       <c r="G40" s="7" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="13" t="n">
         <v>46335</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1285,7 +1698,7 @@
       <c r="G41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="13" t="n">
         <v>46336</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1303,7 +1716,7 @@
       <c r="G42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="13" t="n">
         <v>46337</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1321,7 +1734,7 @@
       <c r="G43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="13" t="n">
         <v>46338</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1339,7 +1752,7 @@
       <c r="G44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="13" t="n">
         <v>46339</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1357,7 +1770,7 @@
       <c r="G45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="14" t="n">
         <v>46340</v>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -1375,7 +1788,7 @@
       <c r="G46" s="7" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="14" t="n">
         <v>46341</v>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -1393,7 +1806,7 @@
       <c r="G47" s="7" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="13" t="n">
         <v>46342</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1411,7 +1824,7 @@
       <c r="G48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="13" t="n">
         <v>46343</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1429,7 +1842,7 @@
       <c r="G49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="13" t="n">
         <v>46344</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1447,7 +1860,7 @@
       <c r="G50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="13" t="n">
         <v>46345</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1465,7 +1878,7 @@
       <c r="G51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="13" t="n">
         <v>46346</v>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1483,7 +1896,7 @@
       <c r="G52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="14" t="n">
         <v>46347</v>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -1501,7 +1914,7 @@
       <c r="G53" s="7" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="n">
+      <c r="A54" s="14" t="n">
         <v>46348</v>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -1519,7 +1932,7 @@
       <c r="G54" s="7" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="13" t="n">
         <v>46349</v>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1537,7 +1950,7 @@
       <c r="G55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="13" t="n">
         <v>46350</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -1555,7 +1968,7 @@
       <c r="G56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="13" t="n">
         <v>46351</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1573,7 +1986,7 @@
       <c r="G57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="13" t="n">
         <v>46352</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1591,7 +2004,7 @@
       <c r="G58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="13" t="n">
         <v>46353</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1609,7 +2022,7 @@
       <c r="G59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="n">
+      <c r="A60" s="14" t="n">
         <v>46354</v>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -1627,7 +2040,7 @@
       <c r="G60" s="7" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="n">
+      <c r="A61" s="14" t="n">
         <v>46355</v>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -1645,7 +2058,7 @@
       <c r="G61" s="7" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="13" t="n">
         <v>46356</v>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1663,7 +2076,7 @@
       <c r="G62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="13" t="n">
         <v>46357</v>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1681,7 +2094,7 @@
       <c r="G63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="13" t="n">
         <v>46358</v>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1699,7 +2112,7 @@
       <c r="G64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="13" t="n">
         <v>46359</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1717,7 +2130,7 @@
       <c r="G65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="13" t="n">
         <v>46360</v>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -1735,7 +2148,7 @@
       <c r="G66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="n">
+      <c r="A67" s="14" t="n">
         <v>46361</v>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -1753,7 +2166,7 @@
       <c r="G67" s="7" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="n">
+      <c r="A68" s="14" t="n">
         <v>46362</v>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -1771,7 +2184,7 @@
       <c r="G68" s="7" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="13" t="n">
         <v>46363</v>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -1789,7 +2202,7 @@
       <c r="G69" s="4" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="13" t="n">
         <v>46364</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -1807,7 +2220,7 @@
       <c r="G70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="13" t="n">
         <v>46365</v>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -1825,7 +2238,7 @@
       <c r="G71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="13" t="n">
         <v>46366</v>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -1843,7 +2256,7 @@
       <c r="G72" s="4" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="13" t="n">
         <v>46367</v>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -1861,7 +2274,7 @@
       <c r="G73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="n">
+      <c r="A74" s="14" t="n">
         <v>46368</v>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -1879,7 +2292,7 @@
       <c r="G74" s="7" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="n">
+      <c r="A75" s="14" t="n">
         <v>46369</v>
       </c>
       <c r="B75" s="6" t="inlineStr">
@@ -1897,7 +2310,7 @@
       <c r="G75" s="7" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="13" t="n">
         <v>46370</v>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -1915,7 +2328,7 @@
       <c r="G76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="13" t="n">
         <v>46371</v>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -1933,7 +2346,7 @@
       <c r="G77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="13" t="n">
         <v>46372</v>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -1951,7 +2364,7 @@
       <c r="G78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="13" t="n">
         <v>46373</v>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -1969,7 +2382,7 @@
       <c r="G79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="13" t="n">
         <v>46374</v>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -1987,7 +2400,7 @@
       <c r="G80" s="4" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="n">
+      <c r="A81" s="14" t="n">
         <v>46375</v>
       </c>
       <c r="B81" s="6" t="inlineStr">
@@ -2005,7 +2418,7 @@
       <c r="G81" s="7" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="n">
+      <c r="A82" s="14" t="n">
         <v>46376</v>
       </c>
       <c r="B82" s="6" t="inlineStr">
@@ -2023,7 +2436,7 @@
       <c r="G82" s="7" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="13" t="n">
         <v>46377</v>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2041,7 +2454,7 @@
       <c r="G83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="13" t="n">
         <v>46378</v>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -2059,7 +2472,7 @@
       <c r="G84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="13" t="n">
         <v>46379</v>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2077,7 +2490,7 @@
       <c r="G85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="13" t="n">
         <v>46380</v>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2095,7 +2508,7 @@
       <c r="G86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="13" t="n">
         <v>46381</v>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2113,7 +2526,7 @@
       <c r="G87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="n">
+      <c r="A88" s="14" t="n">
         <v>46382</v>
       </c>
       <c r="B88" s="6" t="inlineStr">
@@ -2131,7 +2544,7 @@
       <c r="G88" s="7" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="n">
+      <c r="A89" s="14" t="n">
         <v>46383</v>
       </c>
       <c r="B89" s="6" t="inlineStr">
@@ -2149,7 +2562,7 @@
       <c r="G89" s="7" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="13" t="n">
         <v>46384</v>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2167,7 +2580,7 @@
       <c r="G90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="13" t="n">
         <v>46385</v>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2185,7 +2598,7 @@
       <c r="G91" s="4" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="13" t="n">
         <v>46386</v>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -2203,7 +2616,7 @@
       <c r="G92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="13" t="n">
         <v>46387</v>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -2221,7 +2634,7 @@
       <c r="G93" s="4" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="13" t="n">
         <v>46388</v>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -2239,7 +2652,7 @@
       <c r="G94" s="4" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="n">
+      <c r="A95" s="14" t="n">
         <v>46389</v>
       </c>
       <c r="B95" s="6" t="inlineStr">
@@ -2257,7 +2670,7 @@
       <c r="G95" s="7" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="n">
+      <c r="A96" s="14" t="n">
         <v>46390</v>
       </c>
       <c r="B96" s="6" t="inlineStr">
@@ -2275,7 +2688,7 @@
       <c r="G96" s="7" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="13" t="n">
         <v>46391</v>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -2293,7 +2706,7 @@
       <c r="G97" s="4" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="13" t="n">
         <v>46392</v>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -2311,7 +2724,7 @@
       <c r="G98" s="4" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="13" t="n">
         <v>46393</v>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2329,7 +2742,7 @@
       <c r="G99" s="4" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="13" t="n">
         <v>46394</v>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -2347,7 +2760,7 @@
       <c r="G100" s="4" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="13" t="n">
         <v>46395</v>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -2365,7 +2778,7 @@
       <c r="G101" s="4" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="n">
+      <c r="A102" s="14" t="n">
         <v>46396</v>
       </c>
       <c r="B102" s="6" t="inlineStr">
@@ -2383,7 +2796,7 @@
       <c r="G102" s="7" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n">
+      <c r="A103" s="14" t="n">
         <v>46397</v>
       </c>
       <c r="B103" s="6" t="inlineStr">
@@ -2401,7 +2814,7 @@
       <c r="G103" s="7" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="13" t="n">
         <v>46398</v>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -2419,7 +2832,7 @@
       <c r="G104" s="4" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="13" t="n">
         <v>46399</v>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -2437,7 +2850,7 @@
       <c r="G105" s="4" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="13" t="n">
         <v>46400</v>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -2455,7 +2868,7 @@
       <c r="G106" s="4" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="13" t="n">
         <v>46401</v>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -2473,7 +2886,7 @@
       <c r="G107" s="4" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="13" t="n">
         <v>46402</v>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -2491,7 +2904,7 @@
       <c r="G108" s="4" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="n">
+      <c r="A109" s="14" t="n">
         <v>46403</v>
       </c>
       <c r="B109" s="6" t="inlineStr">
@@ -2509,7 +2922,7 @@
       <c r="G109" s="7" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="n">
+      <c r="A110" s="14" t="n">
         <v>46404</v>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -2527,7 +2940,7 @@
       <c r="G110" s="7" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="13" t="n">
         <v>46405</v>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -2545,7 +2958,7 @@
       <c r="G111" s="4" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="13" t="n">
         <v>46406</v>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -2563,7 +2976,7 @@
       <c r="G112" s="4" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="13" t="n">
         <v>46407</v>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -2581,7 +2994,7 @@
       <c r="G113" s="4" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="13" t="n">
         <v>46408</v>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -2599,7 +3012,7 @@
       <c r="G114" s="4" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="13" t="n">
         <v>46409</v>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -2617,7 +3030,7 @@
       <c r="G115" s="4" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="n">
+      <c r="A116" s="14" t="n">
         <v>46410</v>
       </c>
       <c r="B116" s="6" t="inlineStr">
@@ -2635,7 +3048,7 @@
       <c r="G116" s="7" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="n">
+      <c r="A117" s="14" t="n">
         <v>46411</v>
       </c>
       <c r="B117" s="6" t="inlineStr">
@@ -2653,7 +3066,7 @@
       <c r="G117" s="7" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="13" t="n">
         <v>46412</v>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -2671,7 +3084,7 @@
       <c r="G118" s="4" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="13" t="n">
         <v>46413</v>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -2689,7 +3102,7 @@
       <c r="G119" s="4" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="13" t="n">
         <v>46414</v>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -2707,7 +3120,7 @@
       <c r="G120" s="4" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="13" t="n">
         <v>46415</v>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -2725,7 +3138,7 @@
       <c r="G121" s="4" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="13" t="n">
         <v>46416</v>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -2743,7 +3156,7 @@
       <c r="G122" s="4" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="n">
+      <c r="A123" s="14" t="n">
         <v>46417</v>
       </c>
       <c r="B123" s="6" t="inlineStr">
@@ -2761,7 +3174,7 @@
       <c r="G123" s="7" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="5" t="n">
+      <c r="A124" s="14" t="n">
         <v>46418</v>
       </c>
       <c r="B124" s="6" t="inlineStr">
@@ -2779,7 +3192,7 @@
       <c r="G124" s="7" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="13" t="n">
         <v>46419</v>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -2797,7 +3210,7 @@
       <c r="G125" s="4" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="13" t="n">
         <v>46420</v>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -2815,7 +3228,7 @@
       <c r="G126" s="4" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="13" t="n">
         <v>46421</v>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -2833,7 +3246,7 @@
       <c r="G127" s="4" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="13" t="n">
         <v>46422</v>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -2851,7 +3264,7 @@
       <c r="G128" s="4" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="13" t="n">
         <v>46423</v>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -2869,7 +3282,7 @@
       <c r="G129" s="4" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="n">
+      <c r="A130" s="14" t="n">
         <v>46424</v>
       </c>
       <c r="B130" s="6" t="inlineStr">
@@ -2887,7 +3300,7 @@
       <c r="G130" s="7" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="n">
+      <c r="A131" s="14" t="n">
         <v>46425</v>
       </c>
       <c r="B131" s="6" t="inlineStr">
@@ -2905,7 +3318,7 @@
       <c r="G131" s="7" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="13" t="n">
         <v>46426</v>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -2923,7 +3336,7 @@
       <c r="G132" s="4" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="13" t="n">
         <v>46427</v>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -2941,7 +3354,7 @@
       <c r="G133" s="4" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="13" t="n">
         <v>46428</v>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -2959,7 +3372,7 @@
       <c r="G134" s="4" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="13" t="n">
         <v>46429</v>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -2977,7 +3390,7 @@
       <c r="G135" s="4" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="13" t="n">
         <v>46430</v>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -2995,7 +3408,7 @@
       <c r="G136" s="4" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="n">
+      <c r="A137" s="14" t="n">
         <v>46431</v>
       </c>
       <c r="B137" s="6" t="inlineStr">
@@ -3013,7 +3426,7 @@
       <c r="G137" s="7" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="n">
+      <c r="A138" s="14" t="n">
         <v>46432</v>
       </c>
       <c r="B138" s="6" t="inlineStr">
@@ -3031,7 +3444,7 @@
       <c r="G138" s="7" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="13" t="n">
         <v>46433</v>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -3049,7 +3462,7 @@
       <c r="G139" s="4" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="13" t="n">
         <v>46434</v>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -3067,7 +3480,7 @@
       <c r="G140" s="4" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="13" t="n">
         <v>46435</v>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -3085,7 +3498,7 @@
       <c r="G141" s="4" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="13" t="n">
         <v>46436</v>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -3103,7 +3516,7 @@
       <c r="G142" s="4" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="13" t="n">
         <v>46437</v>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -3121,7 +3534,7 @@
       <c r="G143" s="4" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="5" t="n">
+      <c r="A144" s="14" t="n">
         <v>46438</v>
       </c>
       <c r="B144" s="6" t="inlineStr">
@@ -3139,7 +3552,7 @@
       <c r="G144" s="7" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="5" t="n">
+      <c r="A145" s="14" t="n">
         <v>46439</v>
       </c>
       <c r="B145" s="6" t="inlineStr">
@@ -3157,7 +3570,7 @@
       <c r="G145" s="7" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="13" t="n">
         <v>46440</v>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -3175,7 +3588,7 @@
       <c r="G146" s="4" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="13" t="n">
         <v>46441</v>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -3193,7 +3606,7 @@
       <c r="G147" s="4" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="13" t="n">
         <v>46442</v>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -3211,7 +3624,7 @@
       <c r="G148" s="4" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="13" t="n">
         <v>46443</v>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -3229,7 +3642,7 @@
       <c r="G149" s="4" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="13" t="n">
         <v>46444</v>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -3247,7 +3660,7 @@
       <c r="G150" s="4" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="n">
+      <c r="A151" s="14" t="n">
         <v>46445</v>
       </c>
       <c r="B151" s="6" t="inlineStr">
@@ -3265,7 +3678,7 @@
       <c r="G151" s="7" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="n">
+      <c r="A152" s="14" t="n">
         <v>46446</v>
       </c>
       <c r="B152" s="6" t="inlineStr">
@@ -3283,7 +3696,7 @@
       <c r="G152" s="7" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="13" t="n">
         <v>46447</v>
       </c>
       <c r="B153" s="3" t="inlineStr">
@@ -3301,7 +3714,7 @@
       <c r="G153" s="4" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="13" t="n">
         <v>46448</v>
       </c>
       <c r="B154" s="3" t="inlineStr">
@@ -3319,7 +3732,7 @@
       <c r="G154" s="4" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="13" t="n">
         <v>46449</v>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -3337,7 +3750,7 @@
       <c r="G155" s="4" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="13" t="n">
         <v>46450</v>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -3355,7 +3768,7 @@
       <c r="G156" s="4" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="13" t="n">
         <v>46451</v>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -3373,7 +3786,7 @@
       <c r="G157" s="4" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="n">
+      <c r="A158" s="14" t="n">
         <v>46452</v>
       </c>
       <c r="B158" s="6" t="inlineStr">
@@ -3391,7 +3804,7 @@
       <c r="G158" s="7" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="5" t="n">
+      <c r="A159" s="14" t="n">
         <v>46453</v>
       </c>
       <c r="B159" s="6" t="inlineStr">
@@ -3409,7 +3822,7 @@
       <c r="G159" s="7" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="13" t="n">
         <v>46454</v>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -3427,7 +3840,7 @@
       <c r="G160" s="4" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="13" t="n">
         <v>46455</v>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -3445,7 +3858,7 @@
       <c r="G161" s="4" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="13" t="n">
         <v>46456</v>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -3463,7 +3876,7 @@
       <c r="G162" s="4" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="13" t="n">
         <v>46457</v>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -3481,7 +3894,7 @@
       <c r="G163" s="4" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="13" t="n">
         <v>46458</v>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -3499,7 +3912,7 @@
       <c r="G164" s="4" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="5" t="n">
+      <c r="A165" s="14" t="n">
         <v>46459</v>
       </c>
       <c r="B165" s="6" t="inlineStr">
@@ -3517,7 +3930,7 @@
       <c r="G165" s="7" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="5" t="n">
+      <c r="A166" s="14" t="n">
         <v>46460</v>
       </c>
       <c r="B166" s="6" t="inlineStr">
@@ -3535,7 +3948,7 @@
       <c r="G166" s="7" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="13" t="n">
         <v>46461</v>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -3553,7 +3966,7 @@
       <c r="G167" s="4" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="13" t="n">
         <v>46462</v>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -3571,7 +3984,7 @@
       <c r="G168" s="4" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="13" t="n">
         <v>46463</v>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -3589,7 +4002,7 @@
       <c r="G169" s="4" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="13" t="n">
         <v>46464</v>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -3607,7 +4020,7 @@
       <c r="G170" s="4" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="13" t="n">
         <v>46465</v>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -3625,7 +4038,7 @@
       <c r="G171" s="4" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="5" t="n">
+      <c r="A172" s="14" t="n">
         <v>46466</v>
       </c>
       <c r="B172" s="6" t="inlineStr">
@@ -3643,7 +4056,7 @@
       <c r="G172" s="7" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="5" t="n">
+      <c r="A173" s="14" t="n">
         <v>46467</v>
       </c>
       <c r="B173" s="6" t="inlineStr">
@@ -3661,7 +4074,7 @@
       <c r="G173" s="7" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="13" t="n">
         <v>46468</v>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -3679,7 +4092,7 @@
       <c r="G174" s="4" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="13" t="n">
         <v>46469</v>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -3697,7 +4110,7 @@
       <c r="G175" s="4" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="13" t="n">
         <v>46470</v>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -3715,7 +4128,7 @@
       <c r="G176" s="4" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="13" t="n">
         <v>46471</v>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -3733,7 +4146,7 @@
       <c r="G177" s="4" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="13" t="n">
         <v>46472</v>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -3751,7 +4164,7 @@
       <c r="G178" s="4" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="n">
+      <c r="A179" s="14" t="n">
         <v>46473</v>
       </c>
       <c r="B179" s="6" t="inlineStr">
@@ -3769,7 +4182,7 @@
       <c r="G179" s="7" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="5" t="n">
+      <c r="A180" s="14" t="n">
         <v>46474</v>
       </c>
       <c r="B180" s="6" t="inlineStr">
@@ -3787,7 +4200,7 @@
       <c r="G180" s="7" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="13" t="n">
         <v>46475</v>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -3805,7 +4218,7 @@
       <c r="G181" s="4" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="13" t="n">
         <v>46476</v>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -3823,7 +4236,7 @@
       <c r="G182" s="4" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="13" t="n">
         <v>46477</v>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -4073,7 +4486,7 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -4168,9 +4581,15 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n">
+        <v>46296</v>
+      </c>
       <c r="C5" s="3" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ポッドキャスト更新 #3 負け癖からの脱却</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
@@ -4179,9 +4598,15 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n">
+        <v>46297</v>
+      </c>
       <c r="C6" s="3" t="n"/>
-      <c r="D6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>YouTubeに届いたコメント（社会人は時間がないから伸びない？→答えはNO）</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
@@ -4190,9 +4615,15 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n">
+        <v>46297</v>
+      </c>
       <c r="C7" s="3" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>個別学習相談に来られる方々からの声（つまり…）</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
@@ -4201,9 +4632,15 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n">
+        <v>46297</v>
+      </c>
       <c r="C8" s="3" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>正しい方向に最短で進める仕組みが必要／IELTS個別学習相談リンク</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
@@ -4212,9 +4649,15 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n">
+        <v>46298</v>
+      </c>
       <c r="C9" s="3" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>今週早速一歩踏み出したみなさま（相談申込みフォーム通知）</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
@@ -4223,9 +4666,15 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n">
+        <v>46298</v>
+      </c>
       <c r="C10" s="3" t="n"/>
-      <c r="D10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>完璧を待っていたら何も始まらない／「気になる」DM誘導</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
@@ -4234,9 +4683,15 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n">
+        <v>46299</v>
+      </c>
       <c r="C11" s="3" t="n"/>
-      <c r="D11" s="4" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>惜しい!! ライティングの勉強法を変えたら伸びる人</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
@@ -4245,9 +4700,15 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n">
+        <v>46299</v>
+      </c>
       <c r="C12" s="3" t="n"/>
-      <c r="D12" s="4" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>評価基準に沿った書き方を知らないから</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
@@ -4256,9 +4717,15 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n">
+        <v>46299</v>
+      </c>
       <c r="C13" s="3" t="n"/>
-      <c r="D13" s="4" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>頑張りどころを間違えなければ／書き方の方法知りたい？（リアクションスタンプ）</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
@@ -4267,9 +4734,15 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C14" s="3" t="n"/>
-      <c r="D14" s="4" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>昨日のリアクションありがとう→3ステップで解説</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
@@ -4278,9 +4751,15 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C15" s="3" t="n"/>
-      <c r="D15" s="4" t="n"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>ステップ1：評価基準に沿ったライティング教材を選ぶ</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
@@ -4289,9 +4768,15 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C16" s="3" t="n"/>
-      <c r="D16" s="4" t="n"/>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>ステップ2：タスクごとの書き方ルールをインプット</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
@@ -4300,9 +4785,15 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C17" s="3" t="n"/>
-      <c r="D17" s="4" t="n"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ステップ3：ルール確認のために書く／受講生の声</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
@@ -4311,9 +4802,15 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C18" s="3" t="n"/>
-      <c r="D18" s="4" t="n"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>動画講座：全9コース・100本以上</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
@@ -4322,9 +4819,15 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C19" s="3" t="n"/>
-      <c r="D19" s="4" t="n"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>1本5分以内／W5.5→6.5受講生インタビューリンク</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
@@ -4333,9 +4836,15 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n">
+        <v>46300</v>
+      </c>
       <c r="C20" s="3" t="n"/>
-      <c r="D20" s="4" t="n"/>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>ライブ告知（日本時間22時〜 タスク2「書くことがない」を解決）</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
@@ -4344,7 +4853,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -4355,7 +4864,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -4366,7 +4875,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -4377,7 +4886,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -4388,7 +4897,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -4399,7 +4908,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -4410,7 +4919,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -4421,7 +4930,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -4432,7 +4941,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -4443,7 +4952,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -4454,7 +4963,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -4465,7 +4974,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -4476,7 +4985,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -4487,7 +4996,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -4498,7 +5007,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -4509,7 +5018,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -4520,7 +5029,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -4531,7 +5040,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -4542,7 +5051,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -4553,7 +5062,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -4564,7 +5073,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -4575,7 +5084,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -4586,7 +5095,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -4597,7 +5106,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -4606,11 +5115,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4720,7 +5230,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -4731,7 +5241,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -4742,7 +5252,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -4753,7 +5263,7 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -4764,7 +5274,7 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -4775,7 +5285,7 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -4786,7 +5296,7 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
@@ -4797,7 +5307,7 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -4808,7 +5318,7 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -4819,7 +5329,7 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -4830,7 +5340,7 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
@@ -4841,7 +5351,7 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -4852,7 +5362,7 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
@@ -4863,7 +5373,7 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
@@ -4874,7 +5384,7 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -4885,7 +5395,7 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -4896,7 +5406,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -4907,7 +5417,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -4918,7 +5428,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -4929,7 +5439,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -4940,7 +5450,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -4951,7 +5461,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -4962,7 +5472,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -4973,7 +5483,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -4984,7 +5494,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -4995,7 +5505,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -5006,7 +5516,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -5017,7 +5527,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -5028,7 +5538,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -5039,7 +5549,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -5050,7 +5560,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -5061,7 +5571,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -5072,7 +5582,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -5083,7 +5593,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -5094,7 +5604,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -5105,7 +5615,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -5116,7 +5626,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -5127,7 +5637,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -5138,7 +5648,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -5149,7 +5659,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -5158,8 +5668,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5272,7 +5782,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -5283,7 +5793,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -5294,7 +5804,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -5305,7 +5815,7 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -5316,7 +5826,7 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -5327,7 +5837,7 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -5338,7 +5848,7 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
@@ -5349,7 +5859,7 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -5360,7 +5870,7 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -5371,7 +5881,7 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -5382,7 +5892,7 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
@@ -5393,7 +5903,7 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -5404,7 +5914,7 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
@@ -5415,7 +5925,7 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
@@ -5426,7 +5936,7 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -5437,7 +5947,7 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -5448,7 +5958,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -5459,7 +5969,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -5470,7 +5980,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -5481,7 +5991,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -5492,7 +6002,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -5503,7 +6013,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -5514,7 +6024,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -5525,7 +6035,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -5536,7 +6046,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -5547,7 +6057,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -5558,7 +6068,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -5569,7 +6079,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -5580,7 +6090,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -5591,7 +6101,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -5602,7 +6112,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -5613,7 +6123,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -5624,7 +6134,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -5635,7 +6145,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -5646,7 +6156,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -5657,7 +6167,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -5668,7 +6178,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -5679,7 +6189,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -5690,7 +6200,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -5701,7 +6211,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -5710,8 +6220,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5824,7 +6334,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -5835,7 +6345,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -5846,7 +6356,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -5857,7 +6367,7 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -5868,7 +6378,7 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -5879,7 +6389,7 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -5890,7 +6400,7 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
@@ -5901,7 +6411,7 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -5912,7 +6422,7 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -5923,7 +6433,7 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -5934,7 +6444,7 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
@@ -5945,7 +6455,7 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -5956,7 +6466,7 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
@@ -5967,7 +6477,7 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
@@ -5978,7 +6488,7 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -5989,7 +6499,7 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -6000,7 +6510,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -6011,7 +6521,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -6022,7 +6532,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -6033,7 +6543,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -6044,7 +6554,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -6055,7 +6565,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -6066,7 +6576,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -6077,7 +6587,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -6088,7 +6598,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -6099,7 +6609,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -6110,7 +6620,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -6121,7 +6631,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -6132,7 +6642,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -6143,7 +6653,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -6154,7 +6664,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -6165,7 +6675,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -6176,7 +6686,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -6187,7 +6697,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -6198,7 +6708,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -6209,7 +6719,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -6220,7 +6730,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -6231,7 +6741,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -6242,7 +6752,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -6253,7 +6763,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -6262,8 +6772,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6376,7 +6886,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -6387,7 +6897,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -6398,7 +6908,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -6409,7 +6919,7 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -6420,7 +6930,7 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -6431,7 +6941,7 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -6442,7 +6952,7 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
@@ -6453,7 +6963,7 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -6464,7 +6974,7 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -6475,7 +6985,7 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -6486,7 +6996,7 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
@@ -6497,7 +7007,7 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -6508,7 +7018,7 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
@@ -6519,7 +7029,7 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
@@ -6530,7 +7040,7 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -6541,7 +7051,7 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -6552,7 +7062,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -6563,7 +7073,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -6574,7 +7084,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -6585,7 +7095,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -6596,7 +7106,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -6607,7 +7117,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -6618,7 +7128,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -6629,7 +7139,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -6640,7 +7150,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -6651,7 +7161,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -6662,7 +7172,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -6673,7 +7183,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -6684,7 +7194,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -6695,7 +7205,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -6706,7 +7216,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -6717,7 +7227,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -6728,7 +7238,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -6739,7 +7249,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -6750,7 +7260,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -6761,7 +7271,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -6772,7 +7282,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -6783,7 +7293,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -6794,7 +7304,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -6805,7 +7315,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -6814,8 +7324,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6928,7 +7438,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -6939,7 +7449,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -6950,7 +7460,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -6961,7 +7471,7 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="n"/>
+      <c r="B8" s="15" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -6972,7 +7482,7 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="n"/>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -6983,7 +7493,7 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -6994,7 +7504,7 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
@@ -7005,7 +7515,7 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -7016,7 +7526,7 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="n"/>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -7027,7 +7537,7 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="n"/>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -7038,7 +7548,7 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="12" t="n"/>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
@@ -7049,7 +7559,7 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -7060,7 +7570,7 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
@@ -7071,7 +7581,7 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="n"/>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
@@ -7082,7 +7592,7 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="n"/>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -7093,7 +7603,7 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="n"/>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
@@ -7104,7 +7614,7 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="12" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="3" t="n"/>
@@ -7115,7 +7625,7 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="n"/>
+      <c r="B22" s="15" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -7126,7 +7636,7 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="12" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -7137,7 +7647,7 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="15" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -7148,7 +7658,7 @@
       <c r="A25" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="3" t="n"/>
@@ -7159,7 +7669,7 @@
       <c r="A26" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -7170,7 +7680,7 @@
       <c r="A27" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="n"/>
+      <c r="B27" s="15" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="3" t="n"/>
@@ -7181,7 +7691,7 @@
       <c r="A28" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="3" t="n"/>
@@ -7192,7 +7702,7 @@
       <c r="A29" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="3" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="3" t="n"/>
@@ -7203,7 +7713,7 @@
       <c r="A30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="n"/>
+      <c r="B30" s="15" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -7214,7 +7724,7 @@
       <c r="A31" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="3" t="n"/>
@@ -7225,7 +7735,7 @@
       <c r="A32" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -7236,7 +7746,7 @@
       <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="15" t="n"/>
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="3" t="n"/>
@@ -7247,7 +7757,7 @@
       <c r="A34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -7258,7 +7768,7 @@
       <c r="A35" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="15" t="n"/>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="3" t="n"/>
@@ -7269,7 +7779,7 @@
       <c r="A36" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="15" t="n"/>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="3" t="n"/>
@@ -7280,7 +7790,7 @@
       <c r="A37" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="15" t="n"/>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -7291,7 +7801,7 @@
       <c r="A38" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -7302,7 +7812,7 @@
       <c r="A39" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="3" t="n"/>
@@ -7313,7 +7823,7 @@
       <c r="A40" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -7324,7 +7834,7 @@
       <c r="A41" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="12" t="n"/>
+      <c r="B41" s="15" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="3" t="n"/>
@@ -7335,7 +7845,7 @@
       <c r="A42" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="n"/>
+      <c r="B42" s="15" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -7346,7 +7856,7 @@
       <c r="A43" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="12" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="3" t="n"/>
@@ -7357,7 +7867,7 @@
       <c r="A44" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -7366,8 +7876,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E44">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>MAX($E$5:$E$44)</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(E5&lt;&gt;"",E5=MAX($E$5:$E$44))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Replace October stories with the 10/1 screenshots as sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016oX5BAioULTkYoqv5bsGKi
</commit_message>
<xml_diff>
--- a/sns_tracking/SNS記録シート.xlsx
+++ b/sns_tracking/SNS記録シート.xlsx
@@ -268,7 +268,7 @@
       <row>5</row>
       <rowOff>76200</rowOff>
     </from>
-    <ext cx="1400175" cy="2476500"/>
+    <ext cx="1371600" cy="2476500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -293,7 +293,7 @@
       <row>6</row>
       <rowOff>76200</rowOff>
     </from>
-    <ext cx="1400175" cy="2476500"/>
+    <ext cx="1362075" cy="2476500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -318,7 +318,7 @@
       <row>7</row>
       <rowOff>76200</rowOff>
     </from>
-    <ext cx="1390650" cy="2476500"/>
+    <ext cx="1400175" cy="2476500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -326,306 +326,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>8</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1381125" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>9</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1381125" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>10</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1381125" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>11</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1381125" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>12</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>13</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>15</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1371600" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>16</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1371600" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>17</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>18</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>76200</colOff>
-      <row>19</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="1390650" cy="2476500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4599,7 +4299,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="4" t="inlineStr">
@@ -4616,7 +4316,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="15" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="4" t="inlineStr">
@@ -4633,7 +4333,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -4649,15 +4349,9 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="15" t="n">
-        <v>46298</v>
-      </c>
+      <c r="B9" s="15" t="n"/>
       <c r="C9" s="3" t="n"/>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>今週早速一歩踏み出したみなさま（相談申込みフォーム通知）</t>
-        </is>
-      </c>
+      <c r="D9" s="4" t="n"/>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
@@ -4666,15 +4360,9 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="15" t="n">
-        <v>46298</v>
-      </c>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="3" t="n"/>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>完璧を待っていたら何も始まらない／「気になる」DM誘導</t>
-        </is>
-      </c>
+      <c r="D10" s="4" t="n"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
@@ -4683,15 +4371,9 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="15" t="n">
-        <v>46299</v>
-      </c>
+      <c r="B11" s="15" t="n"/>
       <c r="C11" s="3" t="n"/>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>惜しい!! ライティングの勉強法を変えたら伸びる人</t>
-        </is>
-      </c>
+      <c r="D11" s="4" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
@@ -4700,15 +4382,9 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="15" t="n">
-        <v>46299</v>
-      </c>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="3" t="n"/>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>評価基準に沿った書き方を知らないから</t>
-        </is>
-      </c>
+      <c r="D12" s="4" t="n"/>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
@@ -4717,15 +4393,9 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="15" t="n">
-        <v>46299</v>
-      </c>
+      <c r="B13" s="15" t="n"/>
       <c r="C13" s="3" t="n"/>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>頑張りどころを間違えなければ／書き方の方法知りたい？（リアクションスタンプ）</t>
-        </is>
-      </c>
+      <c r="D13" s="4" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
@@ -4734,15 +4404,9 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B14" s="15" t="n"/>
       <c r="C14" s="3" t="n"/>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>昨日のリアクションありがとう→3ステップで解説</t>
-        </is>
-      </c>
+      <c r="D14" s="4" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
@@ -4751,15 +4415,9 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B15" s="15" t="n"/>
       <c r="C15" s="3" t="n"/>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>ステップ1：評価基準に沿ったライティング教材を選ぶ</t>
-        </is>
-      </c>
+      <c r="D15" s="4" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
@@ -4768,15 +4426,9 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B16" s="15" t="n"/>
       <c r="C16" s="3" t="n"/>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>ステップ2：タスクごとの書き方ルールをインプット</t>
-        </is>
-      </c>
+      <c r="D16" s="4" t="n"/>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
@@ -4785,15 +4437,9 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="3" t="n"/>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>ステップ3：ルール確認のために書く／受講生の声</t>
-        </is>
-      </c>
+      <c r="D17" s="4" t="n"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
@@ -4802,15 +4448,9 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B18" s="15" t="n"/>
       <c r="C18" s="3" t="n"/>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>動画講座：全9コース・100本以上</t>
-        </is>
-      </c>
+      <c r="D18" s="4" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
@@ -4819,15 +4459,9 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B19" s="15" t="n"/>
       <c r="C19" s="3" t="n"/>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>1本5分以内／W5.5→6.5受講生インタビューリンク</t>
-        </is>
-      </c>
+      <c r="D19" s="4" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
@@ -4836,15 +4470,9 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="15" t="n">
-        <v>46300</v>
-      </c>
+      <c r="B20" s="15" t="n"/>
       <c r="C20" s="3" t="n"/>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>ライブ告知（日本時間22時〜 タスク2「書くことがない」を解決）</t>
-        </is>
-      </c>
+      <c r="D20" s="4" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>

</xml_diff>

<commit_message>
Add 10/2 story screenshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016oX5BAioULTkYoqv5bsGKi
</commit_message>
<xml_diff>
--- a/sns_tracking/SNS記録シート.xlsx
+++ b/sns_tracking/SNS記録シート.xlsx
@@ -336,6 +336,56 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>8</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1400175" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>76200</colOff>
+      <row>9</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1381125" cy="2476500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -4349,9 +4399,15 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="15" t="n"/>
+      <c r="B9" s="15" t="n">
+        <v>46297</v>
+      </c>
       <c r="C9" s="3" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>今週早速一歩踏み出したみなさま（相談申込みフォーム通知）</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
@@ -4360,9 +4416,15 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="15" t="n"/>
+      <c r="B10" s="15" t="n">
+        <v>46297</v>
+      </c>
       <c r="C10" s="3" t="n"/>
-      <c r="D10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>完璧を待っていたら何も始まらない／「気になる」DM誘導</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>

</xml_diff>